<commit_message>
Update DateBase/orders/Dang Nguyen 195_2026-10-21.xlsx
</commit_message>
<xml_diff>
--- a/DateBase/orders/Dang Nguyen 195_2026-10-21.xlsx
+++ b/DateBase/orders/Dang Nguyen 195_2026-10-21.xlsx
@@ -512,6 +512,9 @@
       <c r="C10" t="str">
         <v>522_山归来绿_Smilax china_undefined_1bunch</v>
       </c>
+      <c r="F10" t="str">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
@@ -570,7 +573,7 @@
         <v>0.00</v>
       </c>
       <c r="G2" t="str">
-        <v>0325255301430100</v>
+        <v>03252553014301015</v>
       </c>
     </row>
   </sheetData>

</xml_diff>